<commit_message>
docs(queue): add implementation report and update WBS for Card 3.12
</commit_message>
<xml_diff>
--- a/docs/Kế hoạch Phân công Dự án EHealth (SRS-EHEALTH-2026-V1).xlsx
+++ b/docs/Kế hoạch Phân công Dự án EHealth (SRS-EHEALTH-2026-V1).xlsx
@@ -1109,7 +1109,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Z36"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="26.38" customWidth="1" style="98" min="1" max="1"/>
     <col width="12" customWidth="1" style="98" min="2" max="2"/>
@@ -2294,15 +2294,15 @@
       </c>
       <c r="H26" s="110" t="inlineStr">
         <is>
-          <t>+ [ ] Tích hợp BullMQ &amp; Redis connection pool vào NestJS server xử lý bất đồng bộ (Section 7.1).
-+ [ ] Queue Workers: email-queue (mail xác nhận, kích hoạt, nhắc hẹn T-24h), sms-queue (OTP, nhắc hẹn T-2h), pdf-queue (sinh PDF đơn thuốc/bệnh án).
-+ [ ] Cấu hình cơ chế Retry tự động (tối đa 3 lần với exponential backoff) khi dịch vụ bên thứ ba gặp sự cố.
-+ [ ] Cron Schedulers: Tự động chuyển lịch hẹn CONFIRMED quá 30 phút thành NO_SHOW vào cuối ngày (Section 5.2); quét dọn dẹp slot giữ chỗ mồ côi.</t>
+          <t>+ [x] Tích hợp BullMQ &amp; Redis connection pool vào NestJS server xử lý bất đồng bộ (Section 7.1).
++ [x] Queue Workers: email-queue (mail xác nhận, kích hoạt, nhắc hẹn T-24h), sms-queue (OTP, nhắc hẹn T-2h), pdf-queue (sinh PDF đơn thuốc/bệnh án).
++ [x] Cấu hình cơ chế Retry tự động (tối đa 3 lần với exponential backoff) khi dịch vụ bên thứ ba gặp sự cố.
++ [x] Cron Schedulers: Tự động chuyển lịch hẹn CONFIRMED quá 30 phút thành NO_SHOW vào cuối ngày (Section 5.2); quét dọn dẹp slot giữ chỗ mồ côi.</t>
         </is>
       </c>
       <c r="I26" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(clinical): [Card 3.5] verify clinical consultation workflow, drug allergy safety and 24h EMR lock
</commit_message>
<xml_diff>
--- a/docs/Kế hoạch Phân công Dự án EHealth (SRS-EHEALTH-2026-V1).xlsx
+++ b/docs/Kế hoạch Phân công Dự án EHealth (SRS-EHEALTH-2026-V1).xlsx
@@ -1109,7 +1109,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Z36"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="26.38" customWidth="1" style="98" min="1" max="1"/>
     <col width="12" customWidth="1" style="98" min="2" max="2"/>
@@ -1983,14 +1983,14 @@
       </c>
       <c r="H19" s="108" t="inlineStr">
         <is>
-          <t>+ [ ] Kiểm thử luồng check-in bằng mã QR tại quầy Lễ tân, kiểm tra đồng bộ realtime lên buồng khám Bác sĩ qua WebSocket (SRS-REC-01).
-+ [ ] Kiểm thử kê đơn thuốc trùng tiền sử dị ứng của bệnh nhân xem popup cảnh báo đỏ có xuất hiện hay không (SRS-DOC-04).
-+ [ ] Kiểm thử bảo mật EMR: Kiểm tra logic chặn sửa đổi bệnh án sau 24 giờ và luồng tạo Addendum (Section 5.4).</t>
+          <t>+ [x] Kiểm thử luồng check-in bằng mã QR tại quầy Lễ tân, kiểm tra đồng bộ realtime lên buồng khám Bác sĩ qua WebSocket (SRS-REC-01).
++ [x] Kiểm thử kê đơn thuốc trùng tiền sử dị ứng của bệnh nhân xem popup cảnh báo đỏ có xuất hiện hay không (SRS-DOC-04).
++ [x] Kiểm thử bảo mật EMR: Kiểm tra logic chặn sửa đổi bệnh án sau 24 giờ và luồng tạo Addendum (Section 5.4).</t>
         </is>
       </c>
       <c r="I19" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(plan): [QA-REVIEW] update plan with Cards 4.9-4.12 and add QA seed script
</commit_message>
<xml_diff>
--- a/docs/Kế hoạch Phân công Dự án EHealth (SRS-EHEALTH-2026-V1).xlsx
+++ b/docs/Kế hoạch Phân công Dự án EHealth (SRS-EHEALTH-2026-V1).xlsx
@@ -12,8 +12,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy, hh:mm"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -1108,7 +1109,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z36"/>
+  <dimension ref="A1:Z40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="26.38" customWidth="1" style="98" min="1" max="1"/>
@@ -2746,6 +2747,182 @@
         </is>
       </c>
       <c r="I36" s="109" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="102" t="n"/>
+      <c r="B37" s="104" t="inlineStr">
+        <is>
+          <t>Card 4.9</t>
+        </is>
+      </c>
+      <c r="C37" s="105" t="inlineStr">
+        <is>
+          <t>[UI/UX] Xây dựng Hệ thống Điều hướng Role-based &amp; Xóa bỏ Trùng lặp 2 Header</t>
+        </is>
+      </c>
+      <c r="D37" s="105" t="inlineStr">
+        <is>
+          <t>🔵 Role: Frontend</t>
+        </is>
+      </c>
+      <c r="E37" s="106" t="inlineStr">
+        <is>
+          <t>1 Người</t>
+        </is>
+      </c>
+      <c r="F37" s="106" t="inlineStr">
+        <is>
+          <t>Lê Việt Cường</t>
+        </is>
+      </c>
+      <c r="G37" s="107" t="n">
+        <v>46296.5</v>
+      </c>
+      <c r="H37" s="110" t="inlineStr">
+        <is>
+          <t>+ [ ] Xóa bỏ Header trùng lặp trong checkin-desk, walkin-booking và phr-profile.
++ [ ] Bổ sung thanh điều hướng nhanh cho Bệnh nhân (Tìm bác sĩ, Lịch sử khám/đơn thuốc, Hồ sơ PHR).
++ [ ] Thêm nút chuyển đổi cho Bác sĩ (Hàng đợi khám &lt;-&gt; Cấu hình ca trực).
++ [ ] Thêm nút chuyển đổi cho Lễ tân (Bàn tiếp đón &lt;-&gt; Tiếp nhận vãng lai).
++ [ ] Xây dựng Sidebar điều hướng cho Admin (Dashboard KPI, Catalogs, Staff, Audit Logs).</t>
+        </is>
+      </c>
+      <c r="I37" s="109" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="102" t="n"/>
+      <c r="B38" s="104" t="inlineStr">
+        <is>
+          <t>Card 4.10</t>
+        </is>
+      </c>
+      <c r="C38" s="105" t="inlineStr">
+        <is>
+          <t>[Auth/UI] Nâng cấp Avatar góc phải: Hiển thị Tên thật, Dropdown Menu &amp; Đăng xuất</t>
+        </is>
+      </c>
+      <c r="D38" s="105" t="inlineStr">
+        <is>
+          <t>🔵 Role: Frontend</t>
+        </is>
+      </c>
+      <c r="E38" s="106" t="inlineStr">
+        <is>
+          <t>1 Người</t>
+        </is>
+      </c>
+      <c r="F38" s="106" t="inlineStr">
+        <is>
+          <t>Lê Việt Cường</t>
+        </is>
+      </c>
+      <c r="G38" s="107" t="n">
+        <v>46296.5</v>
+      </c>
+      <c r="H38" s="110" t="inlineStr">
+        <is>
+          <t>+ [ ] Thay thế icon tĩnh TN bằng Initials Avatar lấy từ tên người dùng thật.
++ [ ] Hiển thị Họ và tên + Badge vai trò của user ở góc trên bên phải Header.
++ [ ] Xây dựng Dropdown Menu khi click Avatar: Bệnh nhân có mục chỉnh sửa Hồ sơ sức khỏe (PHR) và Lịch sử khám; các role khác có lối tắt nhanh.
++ [ ] Tích hợp nút Đăng xuất (Logout) chuẩn trên cả 4 vai trò.</t>
+        </is>
+      </c>
+      <c r="I38" s="109" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="102" t="n"/>
+      <c r="B39" s="104" t="inlineStr">
+        <is>
+          <t>Card 4.11</t>
+        </is>
+      </c>
+      <c r="C39" s="105" t="inlineStr">
+        <is>
+          <t>[Reception] Hoàn thiện Điều hướng 2 chiều cho Bảng gọi số sảnh chờ Smart TV</t>
+        </is>
+      </c>
+      <c r="D39" s="105" t="inlineStr">
+        <is>
+          <t>🔵 Role: Frontend</t>
+        </is>
+      </c>
+      <c r="E39" s="106" t="inlineStr">
+        <is>
+          <t>1 Người</t>
+        </is>
+      </c>
+      <c r="F39" s="106" t="inlineStr">
+        <is>
+          <t>Lê Việt Cường</t>
+        </is>
+      </c>
+      <c r="G39" s="107" t="n">
+        <v>46296.5</v>
+      </c>
+      <c r="H39" s="110" t="inlineStr">
+        <is>
+          <t>+ [ ] Thêm nút mở Bảng gọi số sảnh chờ (Smart TV) tại quầy làm việc của Lễ tân.
++ [ ] Bổ sung nút quay lại quầy lễ tân trên popup Sẵn sàng hiển thị bảng gọi số.
++ [ ] Bổ sung nút/icon Thoát chế độ trình chiếu trên thanh tiêu đề bảng gọi số.</t>
+        </is>
+      </c>
+      <c r="I39" s="109" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="102" t="n"/>
+      <c r="B40" s="104" t="inlineStr">
+        <is>
+          <t>Card 4.12</t>
+        </is>
+      </c>
+      <c r="C40" s="105" t="inlineStr">
+        <is>
+          <t>[Fullstack] Bổ sung Tính năng Upload Avatar và Kênh thông báo Web Push theo SRS</t>
+        </is>
+      </c>
+      <c r="D40" s="105" t="inlineStr">
+        <is>
+          <t>🟣 Role: Fullstack</t>
+        </is>
+      </c>
+      <c r="E40" s="106" t="inlineStr">
+        <is>
+          <t>1 Người</t>
+        </is>
+      </c>
+      <c r="F40" s="106" t="inlineStr">
+        <is>
+          <t>Lê Việt Cường</t>
+        </is>
+      </c>
+      <c r="G40" s="107" t="n">
+        <v>46296.70833333334</v>
+      </c>
+      <c r="H40" s="110" t="inlineStr">
+        <is>
+          <t>+ [ ] Thêm cột avatar_url vào bảng users &amp; doctors; tạo API upload ảnh chân dung (Multer).
++ [ ] Thêm UI upload ảnh tại trang Hồ sơ bệnh nhân (/patient/profile) và form thêm bác sĩ của Admin (/admin/staff).
++ [ ] Hiển thị avatar thật của từng bác sĩ trên doctor-search và booking-stepper.
++ [ ] Tích hợp Web Push API (Service Worker frontend + web-push / VAPID keys backend) hoàn thiện đủ 3 kênh thông báo (Email, SMS, Web Push) theo SRS-PAT-05.</t>
+        </is>
+      </c>
+      <c r="I40" s="109" t="inlineStr">
         <is>
           <t>Chưa bắt đầu</t>
         </is>

</xml_diff>

<commit_message>
docs(tasks): synchronize comprehensive task lists and sprint 4 card statuses
</commit_message>
<xml_diff>
--- a/docs/Kế hoạch Phân công Dự án EHealth (SRS-EHEALTH-2026-V1).xlsx
+++ b/docs/Kế hoạch Phân công Dự án EHealth (SRS-EHEALTH-2026-V1).xlsx
@@ -514,7 +514,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -834,6 +834,7 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1109,7 +1110,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z40"/>
+  <dimension ref="A1:Z43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="26.38" customWidth="1" style="98" min="1" max="1"/>
@@ -1213,7 +1214,7 @@
       </c>
       <c r="I2" s="12" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="Z2" s="5" t="n"/>
@@ -1257,7 +1258,7 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1306,7 @@
       </c>
       <c r="I4" s="26" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1350,7 @@
       </c>
       <c r="I5" s="33" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1395,7 @@
       </c>
       <c r="I6" s="33" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1440,7 @@
       </c>
       <c r="I7" s="33" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1483,7 @@
       </c>
       <c r="I8" s="39" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1534,7 @@
       </c>
       <c r="I9" s="46" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1578,7 @@
       </c>
       <c r="I10" s="52" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1624,7 @@
       </c>
       <c r="I11" s="52" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1669,7 @@
       </c>
       <c r="I12" s="52" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1715,7 @@
       </c>
       <c r="I13" s="52" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1759,7 @@
       </c>
       <c r="I14" s="58" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1810,7 @@
       </c>
       <c r="I15" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1855,7 @@
       </c>
       <c r="I16" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1901,7 @@
       </c>
       <c r="I17" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1949,7 @@
       </c>
       <c r="I18" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2037,7 @@
       </c>
       <c r="I20" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2083,7 @@
       </c>
       <c r="I21" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2128,7 @@
       </c>
       <c r="I22" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2172,7 @@
       </c>
       <c r="I23" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2215,7 +2216,7 @@
       </c>
       <c r="I24" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2260,7 @@
       </c>
       <c r="I25" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2304,7 @@
       </c>
       <c r="I26" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2348,7 @@
       </c>
       <c r="I27" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2392,7 @@
       </c>
       <c r="I28" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2441,7 @@
       </c>
       <c r="I29" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2484,7 @@
       </c>
       <c r="I30" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2529,7 @@
       </c>
       <c r="I31" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2573,7 @@
       </c>
       <c r="I32" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2616,7 +2617,7 @@
       </c>
       <c r="I33" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2660,7 @@
       </c>
       <c r="I34" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang triển khai</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2705,7 @@
       </c>
       <c r="I35" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang triển khai</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2749,7 @@
       </c>
       <c r="I36" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang triển khai</t>
         </is>
       </c>
     </row>
@@ -2793,7 +2794,7 @@
       </c>
       <c r="I37" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2838,7 @@
       </c>
       <c r="I38" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2881,7 @@
       </c>
       <c r="I39" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2925,151 @@
       </c>
       <c r="I40" s="109" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Card 4.13</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>[QA / Hotfix] Xử lý 15 Lỗi Tích hợp &amp; Làm giàu Dữ liệu Seed 625 Slots Khám (BUG-01 -&gt; BUG-15)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>🟣 Role: Fullstack &amp; QA</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1 Người</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Lê Việt Cường</t>
+        </is>
+      </c>
+      <c r="G41" s="111" t="n">
+        <v>46295.95833333334</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>+ [x] Bổ sung Unicode NFD và lọc ngày khám trong doctor-search (BUG-01).
++ [x] Cấu hình chính thức VNPAY Sandbox TMN_CODE &amp; SECRET (BUG-02).
++ [x] Bắt mã hủy MoMo/VNPAY, dừng polling vô hạn, hiển thị màn hình recoverable (BUG-03).
++ [x] Hỗ trợ PATCH /api/v1/phr/me (BUG-04).
++ [x] Gắn RolesGuard cho UserController avatar upload (BUG-05).
++ [x] Sửa Brand Logo routerLink theo dynamic homeRoute() (BUG-06).
++ [x] Đồng bộ thông tin currentUser từ auth session và JWT token lên Header (BUG-07).
++ [x] Sandbox fallback cho OTP SMS logger (BUG-08).
++ [x] Form đặt lịch khám: Tùy chọn đặt cho bản thân và đặt cho người thân (BUG-09).
++ [x] Seed data: 6 chuyên khoa, 6 phòng khám, 5 bác sĩ, 625 slots 3 ca/ngày (BUG-10).
++ [x] Xóa bỏ các header nội bộ trùng lặp (BUG-11).
++ [x] Ẩn header website trên màn hình Smart TV /receptionist/queue-board (BUG-12).
++ [x] Xóa mock 9 bệnh nhân, kết nối API &amp; WebSocket thật cho hàng đợi bác sĩ (BUG-13).
++ [x] Đấu nối hàm Lưu nháp bệnh án (saveDraft) vào CSDL PostgreSQL (BUG-14).
++ [x] Modal xác nhận và sinh chữ ký số SHA-256 khi Hoàn thành ca khám (BUG-15).</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Card 4.14</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>[QA / Hotfix] Khắc phục Toàn diện Lỗi Nghiệp vụ Bác sĩ &amp; Admin Staff theo Báo cáo Rà soát (Thi.docx &amp; Thi (1).docx)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>🟣 Role: Fullstack &amp; QA</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1 Người</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Lê Việt Cường</t>
+        </is>
+      </c>
+      <c r="G42" s="111" t="n">
+        <v>46296.33333333334</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>+ [x] Admin Staff: Bắt lỗi trùng số điện thoại (409 Conflict), hiển thị thông báo lỗi thân thiện thay vì crash.
++ [x] Admin Staff: Khắc phục lỗi reload trang bị mất nhân sự (đồng bộ role trong bảng users và doctors/receptionists).
++ [x] Doctor Schedule: Đấu nối trang cấu hình ca trực Bác sĩ vào PostgreSQL thật qua API /api/v1/doctor/schedules.
++ [x] Admin Staff: Bổ sung trường Giá khám (consultationFee) cho bác sĩ và hiển thị trên màn hình tìm kiếm.
++ [x] Doctor Search: Khắc phục tìm kiếm bác sĩ chuyên khoa Nhi.
++ [x] ICD-10 &amp; Thuốc: Nạp động từ bảng icd10_catalogs và medicines vào buồng khám EMR, xóa bỏ mảng tĩnh DRUGS/ICD.
++ [x] Clinical Summary: Sửa lỗi 403 Forbidden khi bác sĩ xem PHR bệnh nhân bằng endpoint patient-summary.</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Card 4.15</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>[Payment / Lifecycle] Hoàn thiện Chu trình VNPAY/MoMo, Đặt cho Người khác &amp; Sửa lỗi Header Trang Login</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>🟣 Role: Fullstack &amp; QA</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1 Người</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Lê Việt Cường</t>
+        </is>
+      </c>
+      <c r="G43" s="111" t="n">
+        <v>46296.375</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>+ [x] Payment Controller: Hỗ trợ linh hoạt cả UUID và merchantTransactionId (PAY...), sửa lỗi 400 khi VNPAY redirect về và nút Hủy giữ chỗ sau khi hủy trên MoMo.
++ [x] Phân hệ Bệnh nhân: Hoàn thiện tính năng Đặt cho người thân (bookingFor: other), lưu bệnh nhân phụ thuộc và cho phép người đặt xem lịch hẹn.
++ [x] Xác thực: Hoàn thiện luồng Quên mật khẩu qua OTP (trang /forgot-password) và bổ sung ô Nhập lại mật khẩu trang Đăng ký.
++ [x] Header Shell: Khắc phục lỗi hiển thị người dùng và menu Admin khi chưa đăng nhập tại trang /login.
++ [x] Tài liệu: Cập nhật toàn diện danh mục thẻ test VNPAY Sandbox chính thức vào README.md.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>